<commit_message>
#23 eSpark BOM 5,10 and 50 Quantity Updated
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.2/BOM/Client BOM_IOT-Button.xlsx
+++ b/Design Files/IoT-Button-v1.2/BOM/Client BOM_IOT-Button.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="175">
   <si>
     <t>Component list</t>
   </si>
@@ -554,7 +554,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -689,6 +689,32 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -933,7 +959,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1093,6 +1119,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1102,7 +1131,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1527,11 +1565,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1569,7 +1607,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="61"/>
+      <c r="M3" s="62"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1588,7 +1626,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="62"/>
+      <c r="M4" s="63"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1607,7 +1645,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="62"/>
+      <c r="M5" s="63"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1622,7 +1660,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="62"/>
+      <c r="M6" s="63"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1637,7 +1675,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="62"/>
+      <c r="M7" s="63"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1652,7 +1690,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="62"/>
+      <c r="M8" s="63"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2513,36 +2551,38 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="56" t="s">
+      <c r="C32" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="36" t="s">
+      <c r="D32" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="37" t="s">
+      <c r="E32" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="F32" s="36" t="s">
+      <c r="F32" s="65" t="s">
         <v>95</v>
       </c>
-      <c r="G32" s="37" t="s">
+      <c r="G32" s="66" t="s">
         <v>117</v>
       </c>
-      <c r="H32" s="36" t="s">
+      <c r="H32" s="65" t="s">
         <v>127</v>
       </c>
-      <c r="I32" s="37" t="s">
+      <c r="I32" s="66" t="s">
         <v>154</v>
       </c>
-      <c r="J32" s="36"/>
-      <c r="K32" s="36">
-        <v>1</v>
-      </c>
-      <c r="L32" s="37">
+      <c r="J32" s="65"/>
+      <c r="K32" s="65">
+        <v>1</v>
+      </c>
+      <c r="L32" s="66">
         <f>K32*5</f>
         <v>5</v>
       </c>
-      <c r="M32" s="36"/>
+      <c r="M32" s="67" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -2830,7 +2870,7 @@
       <c r="I40" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="J40" s="63" t="s">
+      <c r="J40" s="60" t="s">
         <v>173</v>
       </c>
       <c r="K40" s="36">
@@ -2869,7 +2909,7 @@
       <c r="I41" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="J41" s="63" t="s">
+      <c r="J41" s="60" t="s">
         <v>173</v>
       </c>
       <c r="K41" s="36">
@@ -2954,11 +2994,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2996,7 +3036,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="61"/>
+      <c r="M3" s="62"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -3015,7 +3055,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="62"/>
+      <c r="M4" s="63"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -3034,7 +3074,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="62"/>
+      <c r="M5" s="63"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -3049,7 +3089,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="62"/>
+      <c r="M6" s="63"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -3064,7 +3104,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="62"/>
+      <c r="M7" s="63"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -3079,7 +3119,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="62"/>
+      <c r="M8" s="63"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3940,36 +3980,38 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="56" t="s">
+      <c r="C32" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="36" t="s">
+      <c r="D32" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="37" t="s">
+      <c r="E32" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="F32" s="36" t="s">
+      <c r="F32" s="65" t="s">
         <v>95</v>
       </c>
-      <c r="G32" s="37" t="s">
+      <c r="G32" s="66" t="s">
         <v>117</v>
       </c>
-      <c r="H32" s="36" t="s">
+      <c r="H32" s="65" t="s">
         <v>127</v>
       </c>
-      <c r="I32" s="37" t="s">
+      <c r="I32" s="66" t="s">
         <v>154</v>
       </c>
-      <c r="J32" s="36"/>
-      <c r="K32" s="36">
-        <v>1</v>
-      </c>
-      <c r="L32" s="37">
+      <c r="J32" s="65"/>
+      <c r="K32" s="65">
+        <v>1</v>
+      </c>
+      <c r="L32" s="66">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="M32" s="36"/>
+      <c r="M32" s="67" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="33" spans="1:13" s="59" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="58"/>
@@ -4257,7 +4299,7 @@
       <c r="I40" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="J40" s="63" t="s">
+      <c r="J40" s="60" t="s">
         <v>173</v>
       </c>
       <c r="K40" s="36">
@@ -4296,7 +4338,7 @@
       <c r="I41" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="J41" s="63" t="s">
+      <c r="J41" s="60" t="s">
         <v>173</v>
       </c>
       <c r="K41" s="36">

</xml_diff>

<commit_message>
#23 Client BOM Peripheral description Corrected
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.2/BOM/Client BOM_IOT-Button.xlsx
+++ b/Design Files/IoT-Button-v1.2/BOM/Client BOM_IOT-Button.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="173">
   <si>
     <t>Component list</t>
   </si>
@@ -523,13 +523,7 @@
     <t>Peripheral</t>
   </si>
   <si>
-    <t>104050 3.7V 2600mAh Li-polymer Battery For GPS MP3 Bluetooth Headset Power Bank Rechargeable Lithium Batteria</t>
-  </si>
-  <si>
     <t>Adaptor</t>
-  </si>
-  <si>
-    <t>5V2A New AC 100V-240V Converter Adapter DC 5V 2A 2000mA Power Supply EU Plug DC 5.5mm x 2.1mm</t>
   </si>
   <si>
     <t>Quantity (2 Boards)</t>
@@ -1122,6 +1116,18 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1130,18 +1136,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1565,11 +1559,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1607,7 +1601,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="62"/>
+      <c r="M3" s="66"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1626,7 +1620,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="63"/>
+      <c r="M4" s="67"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1645,7 +1639,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="63"/>
+      <c r="M5" s="67"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1660,7 +1654,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="63"/>
+      <c r="M6" s="67"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1675,7 +1669,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="63"/>
+      <c r="M7" s="67"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1690,7 +1684,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="63"/>
+      <c r="M8" s="67"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1719,7 +1713,7 @@
         <v>162</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K9" s="29" t="s">
         <v>156</v>
@@ -2551,36 +2545,36 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="64" t="s">
+      <c r="C32" s="61" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="65" t="s">
+      <c r="D32" s="62" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="66" t="s">
+      <c r="E32" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="F32" s="65" t="s">
+      <c r="F32" s="62" t="s">
         <v>95</v>
       </c>
-      <c r="G32" s="66" t="s">
+      <c r="G32" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="H32" s="65" t="s">
+      <c r="H32" s="62" t="s">
         <v>127</v>
       </c>
-      <c r="I32" s="66" t="s">
+      <c r="I32" s="63" t="s">
         <v>154</v>
       </c>
-      <c r="J32" s="65"/>
-      <c r="K32" s="65">
-        <v>1</v>
-      </c>
-      <c r="L32" s="66">
+      <c r="J32" s="62"/>
+      <c r="K32" s="62">
+        <v>1</v>
+      </c>
+      <c r="L32" s="63">
         <f>K32*5</f>
         <v>5</v>
       </c>
-      <c r="M32" s="67" t="s">
+      <c r="M32" s="64" t="s">
         <v>154</v>
       </c>
     </row>
@@ -2856,7 +2850,7 @@
         <v>166</v>
       </c>
       <c r="E40" s="36" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F40" s="36" t="s">
         <v>160</v>
@@ -2871,7 +2865,7 @@
         <v>160</v>
       </c>
       <c r="J40" s="60" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K40" s="36">
         <v>1</v>
@@ -2889,13 +2883,13 @@
         <v>32</v>
       </c>
       <c r="C41" s="56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D41" s="36" t="s">
         <v>166</v>
       </c>
       <c r="E41" s="36" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F41" s="36" t="s">
         <v>160</v>
@@ -2910,7 +2904,7 @@
         <v>160</v>
       </c>
       <c r="J41" s="60" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K41" s="36">
         <v>1</v>
@@ -2994,11 +2988,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3036,7 +3030,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="62"/>
+      <c r="M3" s="66"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -3055,7 +3049,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="63"/>
+      <c r="M4" s="67"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -3074,7 +3068,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="63"/>
+      <c r="M5" s="67"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -3089,7 +3083,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="63"/>
+      <c r="M6" s="67"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -3104,7 +3098,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="63"/>
+      <c r="M7" s="67"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -3119,7 +3113,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="63"/>
+      <c r="M8" s="67"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3148,13 +3142,13 @@
         <v>162</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K9" s="29" t="s">
         <v>156</v>
       </c>
       <c r="L9" s="51" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="M9" s="29" t="s">
         <v>164</v>
@@ -3980,36 +3974,36 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="64" t="s">
+      <c r="C32" s="61" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="65" t="s">
+      <c r="D32" s="62" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="66" t="s">
+      <c r="E32" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="F32" s="65" t="s">
+      <c r="F32" s="62" t="s">
         <v>95</v>
       </c>
-      <c r="G32" s="66" t="s">
+      <c r="G32" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="H32" s="65" t="s">
+      <c r="H32" s="62" t="s">
         <v>127</v>
       </c>
-      <c r="I32" s="66" t="s">
+      <c r="I32" s="63" t="s">
         <v>154</v>
       </c>
-      <c r="J32" s="65"/>
-      <c r="K32" s="65">
-        <v>1</v>
-      </c>
-      <c r="L32" s="66">
+      <c r="J32" s="62"/>
+      <c r="K32" s="62">
+        <v>1</v>
+      </c>
+      <c r="L32" s="63">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="M32" s="67" t="s">
+      <c r="M32" s="64" t="s">
         <v>154</v>
       </c>
     </row>
@@ -4272,7 +4266,7 @@
       </c>
       <c r="M39" s="38"/>
     </row>
-    <row r="40" spans="1:13" s="59" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" s="59" customFormat="1" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="58"/>
       <c r="B40" s="50">
         <f t="shared" si="0"/>
@@ -4285,7 +4279,7 @@
         <v>166</v>
       </c>
       <c r="E40" s="36" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F40" s="36" t="s">
         <v>160</v>
@@ -4300,7 +4294,7 @@
         <v>160</v>
       </c>
       <c r="J40" s="60" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K40" s="36">
         <v>1</v>
@@ -4311,20 +4305,20 @@
       </c>
       <c r="M40" s="36"/>
     </row>
-    <row r="41" spans="1:13" s="59" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" s="59" customFormat="1" ht="84.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="58"/>
       <c r="B41" s="50">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D41" s="36" t="s">
         <v>166</v>
       </c>
       <c r="E41" s="36" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F41" s="36" t="s">
         <v>160</v>
@@ -4339,7 +4333,7 @@
         <v>160</v>
       </c>
       <c r="J41" s="60" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K41" s="36">
         <v>1</v>

</xml_diff>